<commit_message>
remove weird whitespace and make sure the numbers are numbers.
</commit_message>
<xml_diff>
--- a/data-raw/juan/battle-assignment1-data.xlsx
+++ b/data-raw/juan/battle-assignment1-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elinwaring/Code/rcode/icorp26/data-raw/juan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{991A6F3B-3791-C348-88DA-12BAB7757D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5CC81004-A7A0-0B49-BA53-CEADA38DAE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="17180" xr2:uid="{3AE9C27F-C084-4F45-8EB1-23A5C85576EE}"/>
   </bookViews>
@@ -192,20 +192,20 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>ID </t>
+      <t>ID</t>
     </r>
   </si>
   <si>
-    <t>Gender </t>
-  </si>
-  <si>
-    <t>Level of Education </t>
-  </si>
-  <si>
-    <t>Age </t>
-  </si>
-  <si>
-    <t>Support for Gun Control </t>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Support for Gun Control</t>
+  </si>
+  <si>
+    <t>Level of Education</t>
+  </si>
+  <si>
+    <t>Age</t>
   </si>
 </sst>
 </file>
@@ -253,10 +253,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -602,522 +603,522 @@
         <v>48</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="A2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="A3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="B5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="B6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="B7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="B8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="2" t="s">
+      <c r="B9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="B10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="B11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="B12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="B13" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="B15" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="B16" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="B17" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="B18" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="B19" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="B20" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="B21" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E22" s="2" t="s">
+      <c r="B22" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="B23" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2" t="s">
+      <c r="B24" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" s="2" t="s">
+      <c r="B25" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E26" s="2" t="s">
+      <c r="B26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="2" t="s">
+      <c r="A27" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D27" s="2" t="s">
+      <c r="B27" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="B28" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="2" t="s">
+      <c r="A29" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="2" t="s">
+      <c r="B29" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E30" s="2" t="s">
+      <c r="B30" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="s">
+      <c r="B31" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="3" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>